<commit_message>
Gap-filling v4b (no stand-in host areas) and v5 (host area as model input); larch/beech host data question
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LTy5LTvQsgDsUNQTkJXWE9
</commit_message>
<xml_diff>
--- a/outputs/tables/QUESTIONS_for_data_providers.xlsx
+++ b/outputs/tables/QUESTIONS_for_data_providers.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -425,51 +425,51 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Forest area total</t>
+          <t>Host data used in the 2025 paper</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Forest appendix vs 2025 paper</t>
+          <t>Paper, Appendix D / Supporting Information</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>The appendix adds up to 87.7 million ha in the reporting regions; the paper gives 102.75 million ha. Which forest area is the paper's figure?</t>
+          <t>The paper compiled host abundance from national forest inventories for Quercus, Fagus, Larix, Picea, Pinus and Abies. Can we have that table? It would give larch and beech their own host data (the forest appendix has neither).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Very large single values</t>
+          <t>Forest area total</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DE DE2 Bavaria, P. abietina (2000-2003)</t>
+          <t>Forest appendix vs 2025 paper</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Pristiphora abietina 58,333 / 76,667 / 113,333 / 200,000 ha in 2000-2003, then 0 from 2004 on. Are these ha defoliated, and are they 3-year averages?</t>
+          <t>The appendix adds up to 87.7 million ha in the reporting regions; the paper gives 102.75 million ha. Which forest area is the paper's figure?</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Every insect reported as 0</t>
+          <t>Very large single values</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AT AT13 (2002)</t>
+          <t>DE DE2 Bavaria, P. abietina (2000-2003)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10 insects reported, all 0 - not monitored, or really no damage?</t>
+          <t>Pristiphora abietina 58,333 / 76,667 / 113,333 / 200,000 ha in 2000-2003, then 0 from 2004 on. Are these ha defoliated, and are they 3-year averages?</t>
         </is>
       </c>
     </row>
@@ -481,12 +481,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DE DE3 (2000-2022)</t>
+          <t>AT AT13 (2002)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
+          <t>10 insects reported, all 0 - not monitored, or really no damage?</t>
         </is>
       </c>
     </row>
@@ -498,7 +498,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DE DE5 (2000-2022)</t>
+          <t>DE DE3 (2000-2022)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -515,7 +515,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DE DE6 (2000-2022)</t>
+          <t>DE DE5 (2000-2022)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -532,7 +532,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DE DE7 (2006-2008, 2011-2022)</t>
+          <t>DE DE6 (2000-2022)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DE DE8 (2022)</t>
+          <t>DE DE7 (2006-2008, 2011-2022)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DE DE9 (2000-2003, 2005-2008, 2010-2015, 2017-2022)</t>
+          <t>DE DE8 (2022)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -583,7 +583,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DE DEE (2007-2008, 2010-2022)</t>
+          <t>DE DE9 (2000-2003, 2005-2008, 2010-2015, 2017-2022)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -600,7 +600,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DE DEF (2004-2006, 2014)</t>
+          <t>DE DEE (2007-2008, 2010-2022)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -612,17 +612,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>Every insect reported as 0</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DE DE1 (2005)</t>
+          <t>DE DEF (2004-2006, 2014)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>pit_cha: 0 vs about 457725 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
         </is>
       </c>
     </row>
@@ -634,12 +634,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DE DE1 (2018)</t>
+          <t>DE DE1 (2005)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>xyl_lin: 0 vs about 120537 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>pit_cha: 0 vs about 457725 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -651,12 +651,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DE DE2 (2007)</t>
+          <t>DE DE1 (2018)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ips_typ: 6000 vs about 4833333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>xyl_lin: 0 vs about 120537 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -668,12 +668,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DE DE2 (2009)</t>
+          <t>DE DE2 (2007)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ips_typ: 3633 vs about 2250000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 6000 vs about 4833333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -685,12 +685,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DE DE2 (2015)</t>
+          <t>DE DE2 (2009)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 3683333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 3633 vs about 2250000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>pit_cha: 0 vs about 316667 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 3683333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -719,12 +719,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DE DE7 (2006)</t>
+          <t>DE DE2 (2015)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 179229 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>pit_cha: 0 vs about 316667 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -736,12 +736,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DE DE8 (2022)</t>
+          <t>DE DE7 (2006)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 266300 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 179229 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>DE DEA (2018)</t>
+          <t>DE DE8 (2022)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 108541 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 266300 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -770,12 +770,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DE DEB; DEC (2005)</t>
+          <t>DE DEA (2018)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>pit_cha: 0 vs about 130961 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 108541 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -787,12 +787,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DE DED (2018)</t>
+          <t>DE DEB; DEC (2005)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ips_sex: 0 vs about 141333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>pit_cha: 0 vs about 130961 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -804,12 +804,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DE DEE (2007)</t>
+          <t>DE DED (2018)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 111370 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_sex: 0 vs about 141333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -821,12 +821,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DE DEF (2002)</t>
+          <t>DE DEE (2007)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ips_ami: 0 vs about 102000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 111370 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -838,12 +838,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DE DEF (2000)</t>
+          <t>DE DEF (2002)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 108000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_ami: 0 vs about 102000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -855,12 +855,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DE DEF (2001)</t>
+          <t>DE DEF (2000)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 200000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 108000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -872,12 +872,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SE SE (2005)</t>
+          <t>DE DEF (2001)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 400000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 200000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SE SE (2012)</t>
+          <t>SE SE (2005)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -906,12 +906,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SE SE (2013)</t>
+          <t>SE SE (2012)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 200000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 400000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -923,29 +923,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SE SE (2017)</t>
+          <t>SE SE (2013)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 1900000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 200000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Values that look like 3-year totals divided by 3</t>
+          <t>Sudden drop to (almost) 0</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>DE DE2 (2000-2022)</t>
+          <t>SE SE (2017)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>227 values, e.g. 15333.33 agr_big - are these multi-year totals divided evenly?</t>
+          <t>ips_typ: 0 vs about 1900000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -957,12 +957,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DE DE7 (2000-2005)</t>
+          <t>DE DE2 (2000-2022)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>20 values, e.g. 66.67 dip_sp - are these multi-year totals divided evenly?</t>
+          <t>227 values, e.g. 15333.33 agr_big - are these multi-year totals divided evenly?</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DE DED (2000-2022)</t>
+          <t>DE DE7 (2000-2005)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>285 values, e.g. 833.33 ips_acu - are these multi-year totals divided evenly?</t>
+          <t>20 values, e.g. 66.67 dip_sp - are these multi-year totals divided evenly?</t>
         </is>
       </c>
     </row>
@@ -991,10 +991,27 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>DE DED (2000-2022)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>285 values, e.g. 833.33 ips_acu - are these multi-year totals divided evenly?</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Values that look like 3-year totals divided by 3</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>DE DEE (2000-2009)</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>95 values, e.g. 416.67 bup_pin - are these multi-year totals divided evenly?</t>
         </is>

</xml_diff>

<commit_message>
WIP: relative damage at all aggregation levels; host check in data questions
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LTy5LTvQsgDsUNQTkJXWE9
</commit_message>
<xml_diff>
--- a/outputs/tables/QUESTIONS_for_data_providers.xlsx
+++ b/outputs/tables/QUESTIONS_for_data_providers.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -476,279 +476,279 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Every insect reported as 0</t>
+          <t>More than 25% of the host in one year</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AT AT13 (2002)</t>
+          <t>PL TOR (2011)</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10 insects reported, all 0 - not monitored, or really no damage?</t>
+          <t>dip_sp:    94,873 ha = 26% of the region's pine forest area in one year. Typing error, wrong unit, or a real outbreak?</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Every insect reported as 0</t>
+          <t>More than 25% of the host in one year</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DE DE3 (2000-2022)</t>
+          <t>PL LUB (2003)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
+          <t>geo_db:    40,984 ha = 35% of the region's broadleaves forest area in one year. Typing error, wrong unit, or a real outbreak?</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Every insect reported as 0</t>
+          <t>More than 25% of the host in one year</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DE DE5 (2000-2022)</t>
+          <t>DE DEF (2018)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
+          <t>ips_typ: 5,670,000 m3 = 54% of the region's spruce growing stock in one year. Typing error, wrong unit, or a real outbreak?</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Every insect reported as 0</t>
+          <t>More than 25% of the host in one year</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DE DE6 (2000-2022)</t>
+          <t>PL LUB (2019)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
+          <t>mel_spp:   176,818 ha = 45% of the region's all forest forest area in one year. Typing error, wrong unit, or a real outbreak?</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Every insect reported as 0</t>
+          <t>More than 25% of the host in one year</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DE DE7 (2006-2008, 2011-2022)</t>
+          <t>CZ CZ02 (2020)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
+          <t>pit_spp:   128,273 m3 = 28% of the region's fir growing stock in one year. Typing error, wrong unit, or a real outbreak?</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Every insect reported as 0</t>
+          <t>More than 25% of the host in one year</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DE DE8 (2022)</t>
+          <t>DE DE2 (2010)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
+          <t>tor_vir:    42,000 ha = 25% of the region's oak forest area in one year. Typing error, wrong unit, or a real outbreak?</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Every insect reported as 0</t>
+          <t>More than 25% of the host in one year</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DE DE9 (2000-2003, 2005-2008, 2010-2015, 2017-2022)</t>
+          <t>DE DE4 (2004)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
+          <t>tor_vir:    18,535 ha = 26% of the region's oak forest area in one year. Typing error, wrong unit, or a real outbreak?</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Every insect reported as 0</t>
+          <t>More than 25% of the host in one year</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DE DEE (2007-2008, 2010-2022)</t>
+          <t>DE DEE (2005)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
+          <t>tor_vir:    15,337 ha = 25% of the region's oak forest area in one year. Typing error, wrong unit, or a real outbreak?</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Every insect reported as 0</t>
+          <t>More than 25% of the host in one year</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DE DEF (2004-2006, 2014)</t>
+          <t>DE DEF (2010)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
+          <t>tor_vir:     6,800 ha = 26% of the region's oak forest area in one year. Typing error, wrong unit, or a real outbreak?</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>More than 25% of the host in one year</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DE DE1 (2005)</t>
+          <t>LT LT (2003)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>pit_cha: 0 vs about 457725 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>tor_vir:    22,895 ha = 67% of the region's oak forest area in one year. Typing error, wrong unit, or a real outbreak?</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>More than 25% of the host in one year</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DE DE1 (2018)</t>
+          <t>PL ZIE (2005)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>xyl_lin: 0 vs about 120537 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>tor_vir:     6,049 ha = 28% of the region's oak forest area in one year. Typing error, wrong unit, or a real outbreak?</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>Every insect reported as 0</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>DE DE2 (2007)</t>
+          <t>AT AT13 (2002)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ips_typ: 6000 vs about 4833333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>10 insects reported, all 0 - not monitored, or really no damage?</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>Every insect reported as 0</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>DE DE2 (2009)</t>
+          <t>DE DE3 (2000-2022)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ips_typ: 3633 vs about 2250000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>Every insect reported as 0</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>DE DE2 (2015)</t>
+          <t>DE DE5 (2000-2022)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 3683333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>Every insect reported as 0</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>DE DE2 (2015)</t>
+          <t>DE DE6 (2000-2022)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>pit_cha: 0 vs about 316667 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>Every insect reported as 0</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DE DE7 (2006)</t>
+          <t>DE DE7 (2006-2008, 2011-2022)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 179229 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>Every insect reported as 0</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -758,58 +758,58 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 266300 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>Every insect reported as 0</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>DE DEA (2018)</t>
+          <t>DE DE9 (2000-2003, 2005-2008, 2010-2015, 2017-2022)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 108541 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>Every insect reported as 0</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DE DEB; DEC (2005)</t>
+          <t>DE DEE (2007-2008, 2010-2022)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>pit_cha: 0 vs about 130961 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Sudden drop to (almost) 0</t>
+          <t>Every insect reported as 0</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DE DED (2018)</t>
+          <t>DE DEF (2004-2006, 2014)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ips_sex: 0 vs about 141333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>44 insects reported, all 0 - not monitored, or really no damage?</t>
         </is>
       </c>
     </row>
@@ -821,12 +821,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>DE DEE (2007)</t>
+          <t>DE DE1 (2005)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 111370 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>pit_cha: 0 vs about 457725 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -838,12 +838,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>DE DEF (2002)</t>
+          <t>DE DE1 (2018)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ips_ami: 0 vs about 102000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>xyl_lin: 0 vs about 120537 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -855,12 +855,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>DE DEF (2000)</t>
+          <t>DE DE2 (2007)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 108000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 6000 vs about 4833333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -872,12 +872,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DE DEF (2001)</t>
+          <t>DE DE2 (2009)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 200000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 3633 vs about 2250000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -889,12 +889,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SE SE (2005)</t>
+          <t>DE DE2 (2015)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 400000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 3683333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -906,12 +906,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SE SE (2012)</t>
+          <t>DE DE2 (2015)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 400000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>pit_cha: 0 vs about 316667 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -923,12 +923,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SE SE (2013)</t>
+          <t>DE DE7 (2006)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 200000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 179229 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
@@ -940,78 +940,265 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SE SE (2017)</t>
+          <t>DE DE8 (2022)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ips_typ: 0 vs about 1900000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+          <t>ips_typ: 0 vs about 266300 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Values that look like 3-year totals divided by 3</t>
+          <t>Sudden drop to (almost) 0</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>DE DE2 (2000-2022)</t>
+          <t>DE DEA (2018)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>227 values, e.g. 15333.33 agr_big - are these multi-year totals divided evenly?</t>
+          <t>ips_typ: 0 vs about 108541 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Values that look like 3-year totals divided by 3</t>
+          <t>Sudden drop to (almost) 0</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>DE DE7 (2000-2005)</t>
+          <t>DE DEB; DEC (2005)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>20 values, e.g. 66.67 dip_sp - are these multi-year totals divided evenly?</t>
+          <t>pit_cha: 0 vs about 130961 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Values that look like 3-year totals divided by 3</t>
+          <t>Sudden drop to (almost) 0</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>DE DED (2000-2022)</t>
+          <t>DE DED (2018)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>285 values, e.g. 833.33 ips_acu - are these multi-year totals divided evenly?</t>
+          <t>ips_sex: 0 vs about 141333 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>Sudden drop to (almost) 0</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>DE DEE (2007)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ips_typ: 0 vs about 111370 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sudden drop to (almost) 0</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>DE DEF (2002)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ips_ami: 0 vs about 102000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Sudden drop to (almost) 0</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>DE DEF (2000)</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ips_typ: 0 vs about 108000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Sudden drop to (almost) 0</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>DE DEF (2001)</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ips_typ: 0 vs about 200000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Sudden drop to (almost) 0</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SE SE (2005)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>ips_typ: 0 vs about 400000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Sudden drop to (almost) 0</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>SE SE (2012)</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>ips_typ: 0 vs about 400000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Sudden drop to (almost) 0</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>SE SE (2013)</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ips_typ: 0 vs about 200000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sudden drop to (almost) 0</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>SE SE (2017)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ips_typ: 0 vs about 1900000 in the years around - typing error (e.g. in 1000 m3) or missing year?</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>Values that look like 3-year totals divided by 3</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>DE DE2 (2000-2022)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>227 values, e.g. 15333.33 agr_big - are these multi-year totals divided evenly?</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Values that look like 3-year totals divided by 3</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>DE DE7 (2000-2005)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>20 values, e.g. 66.67 dip_sp - are these multi-year totals divided evenly?</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Values that look like 3-year totals divided by 3</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>DE DED (2000-2022)</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>285 values, e.g. 833.33 ips_acu - are these multi-year totals divided evenly?</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Values that look like 3-year totals divided by 3</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
         <is>
           <t>DE DEE (2000-2009)</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>95 values, e.g. 416.67 bup_pin - are these multi-year totals divided evenly?</t>
         </is>

</xml_diff>